<commit_message>
redesign for the new sample
</commit_message>
<xml_diff>
--- a/tmp/output.xlsx
+++ b/tmp/output.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:V11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,518 +407,749 @@
         <v>category</v>
       </c>
       <c r="C1" t="str">
-        <v>phone</v>
+        <v>business_phone</v>
       </c>
       <c r="D1" t="str">
-        <v>public_email</v>
+        <v>business_email</v>
       </c>
       <c r="E1" t="str">
         <v>website_url</v>
       </c>
       <c r="F1" t="str">
+        <v>shop_product_count</v>
+      </c>
+      <c r="G1" t="str">
+        <v>meta_ad_count</v>
+      </c>
+      <c r="H1" t="str">
+        <v>revenue_opportunities</v>
+      </c>
+      <c r="I1" t="str">
+        <v>instagram_link</v>
+      </c>
+      <c r="J1" t="str">
+        <v>instagram_desc</v>
+      </c>
+      <c r="K1" t="str">
+        <v>instagram_followers</v>
+      </c>
+      <c r="L1" t="str">
+        <v>instagram_verified</v>
+      </c>
+      <c r="M1" t="str">
+        <v>instagram_engagement_score</v>
+      </c>
+      <c r="N1" t="str">
+        <v>facebook_link</v>
+      </c>
+      <c r="O1" t="str">
+        <v>facebook_reviews</v>
+      </c>
+      <c r="P1" t="str">
+        <v>ecommerce_platform</v>
+      </c>
+      <c r="Q1" t="str">
         <v>website_monthly_visitors</v>
       </c>
-      <c r="G1" t="str">
-        <v>ecom_platform</v>
-      </c>
-      <c r="H1" t="str">
-        <v>meta_ad_count</v>
-      </c>
-      <c r="I1" t="str">
-        <v>fb_link</v>
-      </c>
-      <c r="J1" t="str">
-        <v>fb_reviews</v>
-      </c>
-      <c r="K1" t="str">
-        <v>ig_link</v>
-      </c>
-      <c r="L1" t="str">
-        <v>ig_verified</v>
-      </c>
-      <c r="M1" t="str">
-        <v>ig_description</v>
-      </c>
-      <c r="N1" t="str">
-        <v>ig_followers</v>
-      </c>
-      <c r="O1" t="str">
-        <v>ig_engagement_score</v>
+      <c r="R1" t="str">
+        <v>estimated_monthly_revenue</v>
+      </c>
+      <c r="S1" t="str">
+        <v>email_marketing_tools</v>
+      </c>
+      <c r="T1" t="str">
+        <v>website_performance_mobile</v>
+      </c>
+      <c r="U1" t="str">
+        <v>website_performance_desktop</v>
+      </c>
+      <c r="V1" t="str">
+        <v>website_performance_details</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nova Clothing</v>
+        <v>Northern Garms</v>
       </c>
       <c r="B2" t="str">
-        <v>Men's clothing store</v>
+        <v>Clothing (Brand)</v>
       </c>
       <c r="C2" t="str">
-        <v>+447734723799</v>
+        <v>+44 7479 082512</v>
       </c>
       <c r="D2" t="str">
-        <v>support@novaclothing.co.uk</v>
+        <v>info@northerngarms.co.uk</v>
       </c>
       <c r="E2" t="str">
-        <v>https://novaclothing.co.uk</v>
-      </c>
-      <c r="F2">
-        <v>63294</v>
+        <v>https://northerngarms.co.uk</v>
+      </c>
+      <c r="F2" t="str">
+        <v>153</v>
       </c>
       <c r="G2" t="str">
+        <v>220</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Improve mobile performance; Improve desktop performance; Optimize web pages;</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://www.instagram.com/northerngarms</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Be sure to tag your purchasesBuy Now Pay Later With @klarna @clearpay_uk No Restocks! Once It’s Gone It’s GONE</v>
+      </c>
+      <c r="K2" t="str">
+        <v>91600</v>
+      </c>
+      <c r="L2" t="str">
+        <v>no</v>
+      </c>
+      <c r="M2" t="str">
+        <v>0.34</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://www.facebook.com/northerngarms</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Not yet rated</v>
+      </c>
+      <c r="P2" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H2">
-        <v>96</v>
-      </c>
-      <c r="I2" t="str">
-        <v>https://www.facebook.com/NovaClothingOnline</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Not yet rated (3 Reviews)</v>
-      </c>
-      <c r="K2" t="str">
-        <v>https://www.instagram.com/nova_clothinguk</v>
-      </c>
-      <c r="L2" t="str">
-        <v>No</v>
-      </c>
-      <c r="M2" t="str">
-        <v>We offer a range of clothing from brands such as Dsquared2, Givenchy, Philipp Plein, Balmain, Alexander McQueen,</v>
-      </c>
-      <c r="N2">
-        <v>122000</v>
-      </c>
-      <c r="O2" t="str">
-        <v>0.06</v>
+      <c r="Q2" t="str">
+        <v>81655</v>
+      </c>
+      <c r="R2" t="str">
+        <v>220000</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Klaviyo</v>
+      </c>
+      <c r="T2" t="str">
+        <v>77.25</v>
+      </c>
+      <c r="U2" t="str">
+        <v>65.25</v>
+      </c>
+      <c r="V2" t="str">
+        <v>{"mobile":{"performance":48,"accessibility":88,"bestPractices":73,"seo":100,"avg":77.25},"desktop":{"performance":0,"accessibility":84,"bestPractices":77,"seo":100,"avg":65.25}}</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Forty Clothing</v>
+        <v>Future Past Clothing</v>
       </c>
       <c r="B3" t="str">
-        <v>Men's clothing store</v>
+        <v>Artist</v>
       </c>
       <c r="C3" t="str">
-        <v>+441414651371</v>
+        <v>+44 1283 440053</v>
       </c>
       <c r="D3" t="str">
-        <v>web@fortyclothing.com</v>
+        <v>info@future-past.co.uk</v>
       </c>
       <c r="E3" t="str">
-        <v>https://fortyclothing.com</v>
-      </c>
-      <c r="F3">
-        <v>54453</v>
+        <v>https://future-past.co.uk</v>
+      </c>
+      <c r="F3" t="str">
+        <v>250</v>
       </c>
       <c r="G3" t="str">
+        <v>1200</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Improve mobile performance; Set up automated email campaigns; Add Instagram Shop;</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://www.instagram.com/futurepastclothing</v>
+      </c>
+      <c r="J3" t="str">
+        <v>We’re decadent without precedent.We rage against the dying of the night. Designed with love, worn with pride.Prepare... more</v>
+      </c>
+      <c r="K3" t="str">
+        <v>11900</v>
+      </c>
+      <c r="L3" t="str">
+        <v>yes</v>
+      </c>
+      <c r="M3" t="str">
+        <v>0.28</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://www.facebook.com/futurepastclothing</v>
+      </c>
+      <c r="O3" t="str">
+        <v xml:space="preserve">98% recommend (34 Reviews)﻿</v>
+      </c>
+      <c r="P3" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H3">
-        <v>630</v>
-      </c>
-      <c r="I3" t="str">
-        <v>https://www.facebook.com/fortyclothing</v>
-      </c>
-      <c r="J3" t="str">
-        <v>100% recommend (368 Reviews)</v>
-      </c>
-      <c r="K3" t="str">
-        <v>https://www.instagram.com/fortyclothing</v>
-      </c>
-      <c r="L3" t="str">
-        <v>No</v>
-      </c>
-      <c r="M3" t="str">
-        <v>📍Unit B12 Glasgow Fort 📍11 Royal Exchange Square, Glasgow📍Unit H1A Silverburn#FortyClothing</v>
-      </c>
-      <c r="N3">
-        <v>45000</v>
-      </c>
-      <c r="O3" t="str">
-        <v>0.74</v>
+      <c r="Q3" t="str">
+        <v>78393</v>
+      </c>
+      <c r="R3" t="str">
+        <v>300000</v>
+      </c>
+      <c r="S3" t="str">
+        <v>NA</v>
+      </c>
+      <c r="T3" t="str">
+        <v>88.5</v>
+      </c>
+      <c r="U3" t="str">
+        <v>95.0</v>
+      </c>
+      <c r="V3" t="str">
+        <v>{"mobile":{"performance":67,"accessibility":87,"bestPractices":100,"seo":100,"avg":88.5},"desktop":{"performance":93,"accessibility":87,"bestPractices":100,"seo":100,"avg":95}}</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Cordings of Piccadilly</v>
+        <v>Black Diamond</v>
       </c>
       <c r="B4" t="str">
-        <v>Clothing store</v>
+        <v>Outdoor &amp; Sporting Goods Company</v>
       </c>
       <c r="C4" t="str">
-        <v>+442077584122</v>
+        <v>Reach via IG/FB</v>
       </c>
       <c r="D4" t="str">
-        <v>shop@cordings.co.uk</v>
+        <v>blackdiamond@blackdiamondequipment.com</v>
       </c>
       <c r="E4" t="str">
-        <v>https://cordings.co.uk</v>
-      </c>
-      <c r="F4">
-        <v>514630</v>
+        <v>https://blackdiamondequipment.com</v>
+      </c>
+      <c r="F4" t="str">
+        <v>250</v>
       </c>
       <c r="G4" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="H4">
-        <v>22</v>
+        <v>6800</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Improve mobile performance; Improve desktop performance;</v>
       </c>
       <c r="I4" t="str">
-        <v>https://www.facebook.com/cordings</v>
+        <v>https://www.instagram.com/blackdiamond</v>
       </c>
       <c r="J4" t="str">
-        <v>100% recommend (40 Reviews)</v>
+        <v>Innovative gear for pursuits on rock, ice, snow &amp; trails.</v>
       </c>
       <c r="K4" t="str">
-        <v>https://www.instagram.com/cordingsofpiccadilly</v>
+        <v>995000</v>
       </c>
       <c r="L4" t="str">
-        <v>No</v>
+        <v>yes</v>
       </c>
       <c r="M4" t="str">
-        <v>Since 1839, Cordings has been part of the sartorial landscape of Britain, from our origins as waterproofers to an iconic</v>
-      </c>
-      <c r="N4">
-        <v>36300</v>
+        <v>0.42</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://www.facebook.com/blackdiamondequipment</v>
       </c>
       <c r="O4" t="str">
-        <v>0.81</v>
+        <v xml:space="preserve">56% recommend (24 Reviews)﻿</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Shopify</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>2221000</v>
+      </c>
+      <c r="R4" t="str">
+        <v>20655000</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Klaviyo, HubSpot</v>
+      </c>
+      <c r="T4" t="str">
+        <v>77.25</v>
+      </c>
+      <c r="U4" t="str">
+        <v>78.75</v>
+      </c>
+      <c r="V4" t="str">
+        <v>{"mobile":{"performance":29,"accessibility":99,"bestPractices":96,"seo":85,"avg":77.25},"desktop":{"performance":39,"accessibility":95,"bestPractices":96,"seo":85,"avg":78.75}}</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>OD's Designer Clothing</v>
+        <v>5Brothers</v>
       </c>
       <c r="B5" t="str">
-        <v>Clothing Company</v>
+        <v>Men's clothing store</v>
       </c>
       <c r="C5" t="str">
-        <v>+441744730985</v>
+        <v>Reach via IG/FB</v>
       </c>
       <c r="D5" t="str">
-        <v>sales@odsdesignerclothing.com</v>
+        <v>contact@5brothersclothing.co.uk</v>
       </c>
       <c r="E5" t="str">
-        <v>https://odsdesignerclothing.com</v>
-      </c>
-      <c r="F5">
-        <v>92690</v>
+        <v>https://5brothersclothing.co.uk</v>
+      </c>
+      <c r="F5" t="str">
+        <v>27</v>
       </c>
       <c r="G5" t="str">
+        <v>6200</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Improve mobile performance; Set up automated email campaigns;</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://www.instagram.com/5brothersclothe</v>
+      </c>
+      <c r="J5" t="str">
+        <v>https://www.5brothersclothing.co.ukMen’s clothing brand</v>
+      </c>
+      <c r="K5" t="str">
+        <v>603</v>
+      </c>
+      <c r="L5" t="str">
+        <v>yes</v>
+      </c>
+      <c r="M5" t="str">
+        <v>0.21</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://www.facebook.com/100063181543499</v>
+      </c>
+      <c r="O5" t="str">
+        <v xml:space="preserve">Not yet rated (0 Reviews)﻿</v>
+      </c>
+      <c r="P5" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H5">
-        <v>13</v>
-      </c>
-      <c r="I5" t="str">
-        <v>https://www.facebook.com/odsclothes</v>
-      </c>
-      <c r="J5" t="str">
-        <v>78% recommend (7 Reviews)</v>
-      </c>
-      <c r="K5" t="str">
-        <v>https://www.instagram.com/ods.designerclothing</v>
-      </c>
-      <c r="L5" t="str">
-        <v>No</v>
-      </c>
-      <c r="M5" t="str">
-        <v>👕Clothing 👟Footwear 👜Accessories👨‍👩‍👧Men, Women &amp; Kids💬Email us for queries🗓️Est 1992🌟 4.6/5</v>
-      </c>
-      <c r="N5">
-        <v>3534</v>
-      </c>
-      <c r="O5" t="str">
-        <v>0.33</v>
+      <c r="Q5" t="str">
+        <v>2931</v>
+      </c>
+      <c r="R5" t="str">
+        <v>5000</v>
+      </c>
+      <c r="S5" t="str">
+        <v>NA</v>
+      </c>
+      <c r="T5" t="str">
+        <v>87.0</v>
+      </c>
+      <c r="U5" t="str">
+        <v>92.0</v>
+      </c>
+      <c r="V5" t="str">
+        <v>{"mobile":{"performance":68,"accessibility":92,"bestPractices":96,"seo":92,"avg":87},"desktop":{"performance":88,"accessibility":92,"bestPractices":96,"seo":92,"avg":92}}</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Love Keep Create</v>
+        <v>Forty Clothing</v>
       </c>
       <c r="B6" t="str">
-        <v>Shopping &amp; retail</v>
+        <v>Men's clothing store</v>
       </c>
       <c r="C6" t="str">
-        <v>+443334449144</v>
+        <v>+44 141 465 1371</v>
       </c>
       <c r="D6" t="str">
-        <v>info@lovekeepcreate.co.uk</v>
+        <v>web@fortyclothing.com</v>
       </c>
       <c r="E6" t="str">
-        <v>https://lovekeepcreate.co.uk</v>
-      </c>
-      <c r="F6">
-        <v>44659</v>
+        <v>https://fortyclothing.com</v>
+      </c>
+      <c r="F6" t="str">
+        <v>250</v>
       </c>
       <c r="G6" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="H6">
-        <v>15</v>
+        <v>630</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Improve mobile performance; Optimize web pages;</v>
       </c>
       <c r="I6" t="str">
-        <v>https://www.facebook.com/lovekeepcreate</v>
+        <v>https://www.instagram.com/fortyclothing</v>
       </c>
       <c r="J6" t="str">
-        <v>100% recommend (894 Reviews)</v>
+        <v>📍Unit B12 Glasgow Fort 📍11 Royal Exchange Square, Glasgow📍Unit H1A Silverburn#FortyClothing</v>
       </c>
       <c r="K6" t="str">
-        <v>https://www.instagram.com/lovekeepcreate</v>
+        <v>45000</v>
       </c>
       <c r="L6" t="str">
-        <v>No</v>
+        <v>no</v>
       </c>
       <c r="M6" t="str">
-        <v>Christmas deadline updates on our website 🎄Memory Bears, blankets, cushions and more! 🧸Creating keepsakes from your...</v>
-      </c>
-      <c r="N6">
-        <v>21200</v>
+        <v>0.35</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://www.facebook.com/fortyclothing</v>
       </c>
       <c r="O6" t="str">
-        <v>0.01</v>
+        <v xml:space="preserve">100% recommend (368 Reviews)﻿</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Shopify</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>54453</v>
+      </c>
+      <c r="R6" t="str">
+        <v>150000</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Klaviyo</v>
+      </c>
+      <c r="T6" t="str">
+        <v>75.5</v>
+      </c>
+      <c r="U6" t="str">
+        <v>0.0</v>
+      </c>
+      <c r="V6" t="str">
+        <v>{"mobile":{"performance":60,"accessibility":80,"bestPractices":77,"seo":85,"avg":75.5},"desktop":{"performance":0,"accessibility":0,"bestPractices":0,"seo":0,"avg":0}}</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>New Forest Clothing Ltd</v>
+        <v>Badger Clothing</v>
       </c>
       <c r="B7" t="str">
-        <v>Clothing (Brand)</v>
+        <v>Clothing store</v>
       </c>
       <c r="C7" t="str">
-        <v>+441725510051</v>
+        <v>+44 1273 722245</v>
       </c>
       <c r="D7" t="str">
-        <v>info@newforestclothing.co.uk</v>
+        <v>Reach via IG/FB</v>
       </c>
       <c r="E7" t="str">
-        <v>https://newforestclothing.co.uk</v>
-      </c>
-      <c r="F7">
-        <v>529502</v>
+        <v>https://badgerclothing.co.uk</v>
+      </c>
+      <c r="F7" t="str">
+        <v>250</v>
       </c>
       <c r="G7" t="str">
+        <v>6</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Improve mobile performance; Improve desktop performance; Set up automated email campaigns;</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://www.instagram.com/badgerclothingbrighton</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Established in 1988 Badger is situated in the heart of Brighton offering a wide variety of clothing brands for Men and... more</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2826</v>
+      </c>
+      <c r="L7" t="str">
+        <v>no</v>
+      </c>
+      <c r="M7" t="str">
+        <v>0.28</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://www.facebook.com/badgerclothing</v>
+      </c>
+      <c r="O7" t="str">
+        <v xml:space="preserve">86% recommend (31 Reviews)﻿</v>
+      </c>
+      <c r="P7" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H7">
-        <v>14</v>
-      </c>
-      <c r="I7" t="str">
-        <v>https://www.facebook.com/newforestclothing</v>
-      </c>
-      <c r="J7" t="str">
-        <v>92% recommend (64 Reviews)</v>
-      </c>
-      <c r="K7" t="str">
-        <v>https://www.instagram.com/newforestclothing</v>
-      </c>
-      <c r="L7" t="str">
-        <v>No</v>
-      </c>
-      <c r="M7" t="str">
-        <v>Country Clothing Retailer, family run business based on the edge of the New Forest, UK.International shipping available...</v>
-      </c>
-      <c r="N7">
-        <v>19000</v>
-      </c>
-      <c r="O7" t="str">
-        <v>0.38</v>
+      <c r="Q7" t="str">
+        <v>21868</v>
+      </c>
+      <c r="R7" t="str">
+        <v>50000</v>
+      </c>
+      <c r="S7" t="str">
+        <v>NA</v>
+      </c>
+      <c r="T7" t="str">
+        <v>82.5</v>
+      </c>
+      <c r="U7" t="str">
+        <v>81.5</v>
+      </c>
+      <c r="V7" t="str">
+        <v>{"mobile":{"performance":53,"accessibility":81,"bestPractices":96,"seo":100,"avg":82.5},"desktop":{"performance":52,"accessibility":78,"bestPractices":96,"seo":100,"avg":81.5}}</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>FINDRA Clothing</v>
+        <v>Sproot Baby</v>
       </c>
       <c r="B8" t="str">
-        <v>Clothing (Brand)</v>
+        <v>Baby &amp; children's clothing store</v>
       </c>
       <c r="C8" t="str">
-        <v>+441896870313</v>
+        <v>Reach via IG/FB</v>
       </c>
       <c r="D8" t="str">
-        <v>hello@findra.co.uk</v>
+        <v>hello@sprootbaby.com</v>
       </c>
       <c r="E8" t="str">
-        <v>https://findraclothing.com</v>
-      </c>
-      <c r="F8">
-        <v>50050</v>
+        <v>https://sprootbaby.com</v>
+      </c>
+      <c r="F8" t="str">
+        <v>43</v>
       </c>
       <c r="G8" t="str">
+        <v>13</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Improve mobile performance; Improve desktop performance;</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://www.instagram.com/sprootbaby</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Helping parents today &amp; the planet tomorrow. 🌱👶🏼🌍Soft, organic cotton baby basics. Wear, send back, reward, upcycle.</v>
+      </c>
+      <c r="K8" t="str">
+        <v>1725</v>
+      </c>
+      <c r="L8" t="str">
+        <v>no</v>
+      </c>
+      <c r="M8" t="str">
+        <v>0.25</v>
+      </c>
+      <c r="N8" t="str">
+        <v>https://www.facebook.com/sprootbabyclothes</v>
+      </c>
+      <c r="O8" t="str">
+        <v xml:space="preserve">Not yet rated (0 Reviews)﻿</v>
+      </c>
+      <c r="P8" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H8">
-        <v>65</v>
-      </c>
-      <c r="I8" t="str">
-        <v>https://www.facebook.com/FINDRAclothing</v>
-      </c>
-      <c r="J8" t="str">
-        <v>96% recommend (19 Reviews)</v>
-      </c>
-      <c r="K8" t="str">
-        <v>https://www.instagram.com/findraclothing</v>
-      </c>
-      <c r="L8" t="str">
-        <v>No</v>
-      </c>
-      <c r="M8" t="str">
-        <v>🌿Stylish, versatile &amp; sustainable clothing  🌿Tag us #inmyFINDRA to feature on our feed🌿Shop the collection👇</v>
-      </c>
-      <c r="N8">
-        <v>16500</v>
-      </c>
-      <c r="O8" t="str">
-        <v>0.26</v>
+      <c r="Q8" t="str">
+        <v>6589</v>
+      </c>
+      <c r="R8" t="str">
+        <v>10000</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Klaviyo</v>
+      </c>
+      <c r="T8" t="str">
+        <v>79.25</v>
+      </c>
+      <c r="U8" t="str">
+        <v>84.0</v>
+      </c>
+      <c r="V8" t="str">
+        <v>{"mobile":{"performance":55,"accessibility":81,"bestPractices":96,"seo":85,"avg":79.25},"desktop":{"performance":73,"accessibility":82,"bestPractices":96,"seo":85,"avg":84}}</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Raging Bull Clothing</v>
+        <v>This is Unfolded</v>
       </c>
       <c r="B9" t="str">
-        <v>Clothing store</v>
+        <v>Shopping &amp; retail</v>
       </c>
       <c r="C9" t="str">
-        <v>+441452301869</v>
+        <v>Reach via IG/FB</v>
       </c>
       <c r="D9" t="str">
-        <v>social@ragingbull.co.uk</v>
+        <v>support@thisisunfolded.com</v>
       </c>
       <c r="E9" t="str">
-        <v>https://ragingbull.co.uk</v>
-      </c>
-      <c r="F9">
-        <v>158376</v>
+        <v>https://thisisunfolded.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>250</v>
       </c>
       <c r="G9" t="str">
+        <v>1900</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Improve mobile performance;</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://www.instagram.com/thisisunfolded</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Waste free clothes loved by 100,000 + womenDesigned by you, made for a better 🌎 Newcastle pop up 15th Nov As seen on ... more</v>
+      </c>
+      <c r="K9" t="str">
+        <v>145000</v>
+      </c>
+      <c r="L9" t="str">
+        <v>yes</v>
+      </c>
+      <c r="M9" t="str">
+        <v>0.35</v>
+      </c>
+      <c r="N9" t="str">
+        <v>https://www.facebook.com/thisisunfolded</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Not yet rated</v>
+      </c>
+      <c r="P9" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H9">
-        <v>55</v>
-      </c>
-      <c r="I9" t="str">
-        <v>https://www.facebook.com/RagingBullClothing</v>
-      </c>
-      <c r="J9" t="str">
-        <v>90% recommend (232 Reviews)</v>
-      </c>
-      <c r="K9" t="str">
-        <v>https://www.instagram.com/ragingbullclothing</v>
-      </c>
-      <c r="L9" t="str">
-        <v>No</v>
-      </c>
-      <c r="M9" t="str">
-        <v>Men's clothing brand with a rugby background.Founded by @philvickery3 🏉 Tag your looks #RagingBullClothing📸Shop now ⬇...</v>
-      </c>
-      <c r="N9">
-        <v>16400</v>
-      </c>
-      <c r="O9" t="str">
-        <v>0.16</v>
+      <c r="Q9" t="str">
+        <v>439051</v>
+      </c>
+      <c r="R9" t="str">
+        <v>1205000</v>
+      </c>
+      <c r="S9" t="str">
+        <v>Klaviyo</v>
+      </c>
+      <c r="T9" t="str">
+        <v>83.25</v>
+      </c>
+      <c r="U9" t="str">
+        <v>91.25</v>
+      </c>
+      <c r="V9" t="str">
+        <v>{"mobile":{"performance":54,"accessibility":91,"bestPractices":96,"seo":92,"avg":83.25},"desktop":{"performance":86,"accessibility":91,"bestPractices":96,"seo":92,"avg":91.25}}</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Tilley and Grace</v>
+        <v>Nova Clothing</v>
       </c>
       <c r="B10" t="str">
-        <v>Women's clothing store</v>
+        <v>Men's clothing store</v>
       </c>
       <c r="C10" t="str">
-        <v>+441728685222</v>
+        <v>+44 7734 723799</v>
       </c>
       <c r="D10" t="str">
-        <v>hello@tilleyandgrace.co.uk</v>
+        <v>support@novaclothing.co.uk</v>
       </c>
       <c r="E10" t="str">
-        <v>https://tilleyandgrace.co.uk</v>
-      </c>
-      <c r="F10">
-        <v>25529</v>
+        <v>https://novaclothing.co.uk</v>
+      </c>
+      <c r="F10" t="str">
+        <v>250</v>
       </c>
       <c r="G10" t="str">
+        <v>96</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Improve mobile performance; Improve desktop performance;</v>
+      </c>
+      <c r="I10" t="str">
+        <v>https://www.instagram.com/nova_clothinguk</v>
+      </c>
+      <c r="J10" t="str">
+        <v>We offer a range of clothing from brands such as Dsquared2, Givenchy, Philipp Plein, Balmain, Alexander McQueen,... more</v>
+      </c>
+      <c r="K10" t="str">
+        <v>122000</v>
+      </c>
+      <c r="L10" t="str">
+        <v>no</v>
+      </c>
+      <c r="M10" t="str">
+        <v>0.35</v>
+      </c>
+      <c r="N10" t="str">
+        <v>https://www.facebook.com/NovaClothingOnline</v>
+      </c>
+      <c r="O10" t="str">
+        <v xml:space="preserve">Not yet rated (3 Reviews)﻿</v>
+      </c>
+      <c r="P10" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H10">
-        <v>25</v>
-      </c>
-      <c r="I10" t="str">
-        <v>https://www.facebook.com/TilleyandGrace</v>
-      </c>
-      <c r="J10" t="str">
-        <v>96% recommend (19 Reviews)</v>
-      </c>
-      <c r="K10" t="str">
-        <v>https://www.instagram.com/tilleyandgrace</v>
-      </c>
-      <c r="L10" t="str">
-        <v>No</v>
-      </c>
-      <c r="M10" t="str">
-        <v>A women’s fashion retailer with a passion for colourAldeburgh | Woodbridge | Southwold | Holt</v>
-      </c>
-      <c r="N10">
-        <v>12100</v>
-      </c>
-      <c r="O10" t="str">
-        <v>0.07</v>
+      <c r="Q10" t="str">
+        <v>63294</v>
+      </c>
+      <c r="R10" t="str">
+        <v>175000</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Klaviyo, Omnisend</v>
+      </c>
+      <c r="T10" t="str">
+        <v>63.25</v>
+      </c>
+      <c r="U10" t="str">
+        <v>75.75</v>
+      </c>
+      <c r="V10" t="str">
+        <v>{"mobile":{"performance":16,"accessibility":91,"bestPractices":54,"seo":92,"avg":63.25},"desktop":{"performance":66,"accessibility":91,"bestPractices":54,"seo":92,"avg":75.75}}</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>FDX Sports &amp; Outdoors</v>
+        <v>Thrivin</v>
       </c>
       <c r="B11" t="str">
-        <v>Brand</v>
+        <v>Clothing (Brand)</v>
       </c>
       <c r="C11" t="str">
-        <v>+442086170050</v>
+        <v>Reach via IG/FB</v>
       </c>
       <c r="D11" t="str">
-        <v>info@fdxsports.co.uk</v>
+        <v>info@thrivin-gymwear.com</v>
       </c>
       <c r="E11" t="str">
-        <v>https://fdxsports.co.uk</v>
-      </c>
-      <c r="F11">
-        <v>24324</v>
+        <v>https://thrivin-gymwear.com</v>
+      </c>
+      <c r="F11" t="str">
+        <v>141</v>
       </c>
       <c r="G11" t="str">
+        <v>720</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Improve mobile performance; Improve desktop performance; Optimize web pages;</v>
+      </c>
+      <c r="I11" t="str">
+        <v>https://www.instagram.com/thrivingymwear</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Because when you believe, you become unstoppable.✨CHIARA X THRIVIN 👀 LAUNCH LIVE NOW.</v>
+      </c>
+      <c r="K11" t="str">
+        <v>85800</v>
+      </c>
+      <c r="L11" t="str">
+        <v>yes</v>
+      </c>
+      <c r="M11" t="str">
+        <v>0.35</v>
+      </c>
+      <c r="N11" t="str">
+        <v>https://www.facebook.com/100066432025945</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Not yet rated</v>
+      </c>
+      <c r="P11" t="str">
         <v>Shopify</v>
       </c>
-      <c r="H11">
-        <v>27</v>
-      </c>
-      <c r="I11" t="str">
-        <v>https://www.facebook.com/fdxsportsuk</v>
-      </c>
-      <c r="J11" t="str">
-        <v>Not yet rated (2 Reviews)</v>
-      </c>
-      <c r="K11" t="str">
-        <v>https://www.instagram.com/fdx_sports</v>
-      </c>
-      <c r="L11" t="str">
-        <v>No</v>
-      </c>
-      <c r="M11" t="str">
-        <v>Embrace your journey, ignite your ride.#fdx #keepriding</v>
-      </c>
-      <c r="N11">
-        <v>2734</v>
-      </c>
-      <c r="O11" t="str">
-        <v>0.33</v>
+      <c r="Q11" t="str">
+        <v>117508</v>
+      </c>
+      <c r="R11" t="str">
+        <v>325000</v>
+      </c>
+      <c r="S11" t="str">
+        <v>Klaviyo</v>
+      </c>
+      <c r="T11" t="str">
+        <v>72.25</v>
+      </c>
+      <c r="U11" t="str">
+        <v>65.5</v>
+      </c>
+      <c r="V11" t="str">
+        <v>{"mobile":{"performance":42,"accessibility":89,"bestPractices":73,"seo":85,"avg":72.25},"desktop":{"performance":0,"accessibility":97,"bestPractices":73,"seo":92,"avg":65.5}}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>